<commit_message>
feat(sales): add Food/Drink sales streams with flexible CSV import
MEP treats Food as editable and Drink as Store−Food auto-calc; CSV import accepts either side and wires PL Analyze sales rows from dailyIncome.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/excel/2026年売上入力用.xlsx
+++ b/excel/2026年売上入力用.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10703"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10713"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/shinmatsushita/Desktop/kpi-navigator/excel/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B1A53981-DEA1-3D41-AE8D-A87DAB09B958}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{808BAB97-4A8E-4F4C-A5BE-2AC0072C86A6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="13480" yWindow="1120" windowWidth="11820" windowHeight="14880" xr2:uid="{8DB7F31A-B26B-8B41-A3DA-61B603341751}"/>
   </bookViews>
@@ -3197,7 +3197,9 @@
       <c r="C196" s="4">
         <v>1</v>
       </c>
-      <c r="D196" s="5"/>
+      <c r="D196" s="5">
+        <v>2549.8395867319196</v>
+      </c>
     </row>
     <row r="197" spans="1:4">
       <c r="A197" s="2">
@@ -3209,7 +3211,9 @@
       <c r="C197" s="4">
         <v>1</v>
       </c>
-      <c r="D197" s="5"/>
+      <c r="D197" s="5">
+        <v>1843.5535617183252</v>
+      </c>
     </row>
     <row r="198" spans="1:4">
       <c r="A198" s="2">
@@ -3221,7 +3225,9 @@
       <c r="C198" s="4">
         <v>1</v>
       </c>
-      <c r="D198" s="5"/>
+      <c r="D198" s="5">
+        <v>2159.6592350915353</v>
+      </c>
     </row>
     <row r="199" spans="1:4">
       <c r="A199" s="2">
@@ -3233,7 +3239,9 @@
       <c r="C199" s="4">
         <v>1</v>
       </c>
-      <c r="D199" s="5"/>
+      <c r="D199" s="5">
+        <v>3049.4870400580025</v>
+      </c>
     </row>
     <row r="200" spans="1:4">
       <c r="A200" s="2">
@@ -3245,7 +3253,9 @@
       <c r="C200" s="4">
         <v>1</v>
       </c>
-      <c r="D200" s="5"/>
+      <c r="D200" s="5">
+        <v>708.8363240891789</v>
+      </c>
     </row>
     <row r="201" spans="1:4">
       <c r="A201" s="2">
@@ -3269,7 +3279,9 @@
       <c r="C202" s="4">
         <v>1</v>
       </c>
-      <c r="D202" s="5"/>
+      <c r="D202" s="5">
+        <v>2961.4962842124341</v>
+      </c>
     </row>
     <row r="203" spans="1:4">
       <c r="A203" s="2">

</xml_diff>